<commit_message>
Sample data: keep August fuel purchases inside the trip period
</commit_message>
<xml_diff>
--- a/sample/Sample_Fuel_Vehicle_Report_August_2026.xlsx
+++ b/sample/Sample_Fuel_Vehicle_Report_August_2026.xlsx
@@ -584,7 +584,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02/08/26</t>
+          <t>03/08/26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -604,7 +604,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>24.20L</t>
+          <t>15.24L</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -613,25 +613,25 @@
         </is>
       </c>
       <c r="G8" s="6" t="n">
-        <v>59.29</v>
+        <v>37.34</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>7.73</v>
+        <v>4.87</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>-0.71</v>
+        <v>-0.45</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>58.58</v>
+        <v>36.89</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>50.94</v>
+        <v>32.08</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03/08/26</t>
+          <t>04/08/26</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>15.24L</t>
+          <t>15.34L</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -660,25 +660,25 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>37.34</v>
+        <v>37.58</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>4.87</v>
+        <v>4.9</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>-0.75</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>36.59</v>
+        <v>36.83</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>31.82</v>
+        <v>32.03</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04/08/26</t>
+          <t>07/08/26</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>15.34L</t>
+          <t>24.20L</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -707,19 +707,19 @@
         </is>
       </c>
       <c r="G10" s="6" t="n">
-        <v>37.58</v>
+        <v>59.29</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>4.9</v>
+        <v>7.73</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>-0</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>37.58</v>
+        <v>59.29</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>32.68</v>
+        <v>51.56</v>
       </c>
     </row>
     <row r="11">
@@ -954,13 +954,13 @@
         <v>40.56</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>-2.13</v>
+        <v>-1.87</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>308.8</v>
+        <v>309.06</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>268.52</v>
+        <v>268.75</v>
       </c>
     </row>
     <row r="18">
@@ -2595,7 +2595,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>02/08/26</t>
+          <t>07/08/26</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>117.22L</t>
+          <t>36.06L</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2624,25 +2624,25 @@
         </is>
       </c>
       <c r="G61" s="6" t="n">
-        <v>327.04</v>
+        <v>100.61</v>
       </c>
       <c r="H61" s="6" t="n">
-        <v>42.66</v>
+        <v>13.12</v>
       </c>
       <c r="I61" s="6" t="n">
         <v>-0</v>
       </c>
       <c r="J61" s="6" t="n">
-        <v>327.04</v>
+        <v>100.61</v>
       </c>
       <c r="K61" s="6" t="n">
-        <v>284.38</v>
+        <v>87.48999999999999</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>07/08/26</t>
+          <t>10/08/26</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2662,7 +2662,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>36.06L</t>
+          <t>117.22L</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2671,19 +2671,19 @@
         </is>
       </c>
       <c r="G62" s="6" t="n">
-        <v>100.61</v>
+        <v>327.04</v>
       </c>
       <c r="H62" s="6" t="n">
-        <v>13.12</v>
+        <v>42.66</v>
       </c>
       <c r="I62" s="6" t="n">
         <v>-0</v>
       </c>
       <c r="J62" s="6" t="n">
-        <v>100.61</v>
+        <v>327.04</v>
       </c>
       <c r="K62" s="6" t="n">
-        <v>87.48999999999999</v>
+        <v>284.38</v>
       </c>
     </row>
     <row r="63">

</xml_diff>

<commit_message>
Sample data: add South Island section to schedule, end period 30 Oct
</commit_message>
<xml_diff>
--- a/sample/Sample_Fuel_Vehicle_Report_August_2026.xlsx
+++ b/sample/Sample_Fuel_Vehicle_Report_August_2026.xlsx
@@ -584,7 +584,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03/08/26</t>
+          <t>02/08/26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -604,7 +604,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>15.24L</t>
+          <t>24.20L</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -613,25 +613,25 @@
         </is>
       </c>
       <c r="G8" s="6" t="n">
-        <v>37.34</v>
+        <v>59.29</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>4.87</v>
+        <v>7.73</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>-0.45</v>
+        <v>-0.71</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>36.89</v>
+        <v>58.58</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>32.08</v>
+        <v>50.94</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04/08/26</t>
+          <t>03/08/26</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>15.34L</t>
+          <t>15.24L</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -660,25 +660,25 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>37.58</v>
+        <v>37.34</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>4.9</v>
+        <v>4.87</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>-0.75</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>36.83</v>
+        <v>36.59</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>32.03</v>
+        <v>31.82</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07/08/26</t>
+          <t>04/08/26</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>24.20L</t>
+          <t>15.34L</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -707,19 +707,19 @@
         </is>
       </c>
       <c r="G10" s="6" t="n">
-        <v>59.29</v>
+        <v>37.58</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>7.73</v>
+        <v>4.9</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>-0</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>59.29</v>
+        <v>37.58</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>51.56</v>
+        <v>32.68</v>
       </c>
     </row>
     <row r="11">
@@ -954,13 +954,13 @@
         <v>40.56</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>-1.87</v>
+        <v>-2.13</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>309.06</v>
+        <v>308.8</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>268.75</v>
+        <v>268.52</v>
       </c>
     </row>
     <row r="18">
@@ -2595,7 +2595,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>07/08/26</t>
+          <t>02/08/26</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>36.06L</t>
+          <t>117.22L</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2624,25 +2624,25 @@
         </is>
       </c>
       <c r="G61" s="6" t="n">
-        <v>100.61</v>
+        <v>327.04</v>
       </c>
       <c r="H61" s="6" t="n">
-        <v>13.12</v>
+        <v>42.66</v>
       </c>
       <c r="I61" s="6" t="n">
         <v>-0</v>
       </c>
       <c r="J61" s="6" t="n">
-        <v>100.61</v>
+        <v>327.04</v>
       </c>
       <c r="K61" s="6" t="n">
-        <v>87.48999999999999</v>
+        <v>284.38</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>10/08/26</t>
+          <t>07/08/26</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2662,7 +2662,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>117.22L</t>
+          <t>36.06L</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2671,19 +2671,19 @@
         </is>
       </c>
       <c r="G62" s="6" t="n">
-        <v>327.04</v>
+        <v>100.61</v>
       </c>
       <c r="H62" s="6" t="n">
-        <v>42.66</v>
+        <v>13.12</v>
       </c>
       <c r="I62" s="6" t="n">
         <v>-0</v>
       </c>
       <c r="J62" s="6" t="n">
-        <v>327.04</v>
+        <v>100.61</v>
       </c>
       <c r="K62" s="6" t="n">
-        <v>284.38</v>
+        <v>87.48999999999999</v>
       </c>
     </row>
     <row r="63">

</xml_diff>

<commit_message>
Sample data: South Island section in schedule
Co-authored-by: Rimsha Shakya <rimshashakya11-dotcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/sample/Sample_Fuel_Vehicle_Report_August_2026.xlsx
+++ b/sample/Sample_Fuel_Vehicle_Report_August_2026.xlsx
@@ -584,7 +584,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03/08/26</t>
+          <t>02/08/26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -604,7 +604,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>15.24L</t>
+          <t>24.20L</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -613,25 +613,25 @@
         </is>
       </c>
       <c r="G8" s="6" t="n">
-        <v>37.34</v>
+        <v>59.29</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>4.87</v>
+        <v>7.73</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>-0.45</v>
+        <v>-0.71</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>36.89</v>
+        <v>58.58</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>32.08</v>
+        <v>50.94</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04/08/26</t>
+          <t>03/08/26</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>15.34L</t>
+          <t>15.24L</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -660,25 +660,25 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>37.58</v>
+        <v>37.34</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>4.9</v>
+        <v>4.87</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>-0.75</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>36.83</v>
+        <v>36.59</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>32.03</v>
+        <v>31.82</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07/08/26</t>
+          <t>04/08/26</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>24.20L</t>
+          <t>15.34L</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -707,19 +707,19 @@
         </is>
       </c>
       <c r="G10" s="6" t="n">
-        <v>59.29</v>
+        <v>37.58</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>7.73</v>
+        <v>4.9</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>-0</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>59.29</v>
+        <v>37.58</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>51.56</v>
+        <v>32.68</v>
       </c>
     </row>
     <row r="11">
@@ -954,13 +954,13 @@
         <v>40.56</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>-1.87</v>
+        <v>-2.13</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>309.06</v>
+        <v>308.8</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>268.75</v>
+        <v>268.52</v>
       </c>
     </row>
     <row r="18">
@@ -2595,7 +2595,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>07/08/26</t>
+          <t>02/08/26</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>36.06L</t>
+          <t>117.22L</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2624,25 +2624,25 @@
         </is>
       </c>
       <c r="G61" s="6" t="n">
-        <v>100.61</v>
+        <v>327.04</v>
       </c>
       <c r="H61" s="6" t="n">
-        <v>13.12</v>
+        <v>42.66</v>
       </c>
       <c r="I61" s="6" t="n">
         <v>-0</v>
       </c>
       <c r="J61" s="6" t="n">
-        <v>100.61</v>
+        <v>327.04</v>
       </c>
       <c r="K61" s="6" t="n">
-        <v>87.48999999999999</v>
+        <v>284.38</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>10/08/26</t>
+          <t>07/08/26</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2662,7 +2662,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>117.22L</t>
+          <t>36.06L</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2671,19 +2671,19 @@
         </is>
       </c>
       <c r="G62" s="6" t="n">
-        <v>327.04</v>
+        <v>100.61</v>
       </c>
       <c r="H62" s="6" t="n">
-        <v>42.66</v>
+        <v>13.12</v>
       </c>
       <c r="I62" s="6" t="n">
         <v>-0</v>
       </c>
       <c r="J62" s="6" t="n">
-        <v>327.04</v>
+        <v>100.61</v>
       </c>
       <c r="K62" s="6" t="n">
-        <v>284.38</v>
+        <v>87.48999999999999</v>
       </c>
     </row>
     <row r="63">

</xml_diff>